<commit_message>
parámetros del modelo del 2018 y 2019
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Comparación chi cuadrado espectros del 2018 y 2019.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Comparación chi cuadrado espectros del 2018 y 2019.xlsx
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4816</v>
+        <v>0.4434</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4508</v>
+        <v>0.4504</v>
       </c>
       <c r="D4" t="n">
         <v>0.9</v>
@@ -523,10 +523,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4017</v>
+        <v>0.4005</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4101</v>
+        <v>0.4074</v>
       </c>
       <c r="D5" t="n">
         <v>0.5</v>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4674</v>
+        <v>0.4815</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5274</v>
+        <v>0.5306</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5415</v>
+        <v>0.5376</v>
       </c>
       <c r="D7" t="n">
         <v>0.4</v>
@@ -584,10 +584,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.415</v>
+        <v>0.4151</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4208</v>
+        <v>0.4201</v>
       </c>
       <c r="D8" t="n">
         <v>0.5</v>
@@ -606,7 +606,7 @@
         <v>0.9725</v>
       </c>
       <c r="C9" t="n">
-        <v>0.985</v>
+        <v>0.9849</v>
       </c>
       <c r="D9" t="n">
         <v>0.4</v>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9368</v>
+        <v>0.9369</v>
       </c>
       <c r="C10" t="n">
         <v>0.9455</v>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.6178</v>
+        <v>2.2336</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
espectros del 2018 y 2019
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Comparación chi cuadrado espectros del 2018 y 2019.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Comparación chi cuadrado espectros del 2018 y 2019.xlsx
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7557</v>
+        <v>0.7564</v>
       </c>
       <c r="C2" t="n">
-        <v>0.763</v>
+        <v>0.7634</v>
       </c>
       <c r="D2" t="n">
         <v>0.7</v>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3863</v>
+        <v>0.3872</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4434</v>
+        <v>0.4442</v>
       </c>
       <c r="C4" t="n">
         <v>0.4504</v>
@@ -523,10 +523,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4005</v>
+        <v>0.4007</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4074</v>
+        <v>0.4096</v>
       </c>
       <c r="D5" t="n">
         <v>0.5</v>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4815</v>
+        <v>0.4697</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5306</v>
+        <v>0.531</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5376</v>
+        <v>0.5448</v>
       </c>
       <c r="D7" t="n">
         <v>0.4</v>
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9725</v>
+        <v>0.975</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9849</v>
+        <v>0.9873</v>
       </c>
       <c r="D9" t="n">
         <v>0.4</v>
@@ -622,10 +622,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9369</v>
+        <v>0.9371</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9455</v>
+        <v>0.9452</v>
       </c>
       <c r="D10" t="n">
         <v>0.5</v>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.2336</v>
+        <v>2.267</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
parametros espectros del 2018 y 2019
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Comparación chi cuadrado espectros del 2018 y 2019.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Comparación chi cuadrado espectros del 2018 y 2019.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,21 +637,67 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Septiembre 21-2018</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.6926</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>No existe</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No existe</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Agosto 05-2019</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>2.267</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>No existe</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+      <c r="B12" t="n">
+        <v>2.7597</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>No existe</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>0.5</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No existe</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Agosto 06-2019</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5.0565</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>No existe</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>No existe</t>
         </is>

</xml_diff>